<commit_message>
Add 90 new industrial biotech facilities (502 total) + auth/admin features
Expands the global database from 412 to 502 facilities, adding Lallemand,
AB Mauri, Ohly, Lesaffre, AB Enzymes, Sensient, Kyowa Hakko Bio, Global
Bio-Chem, Vedan, Zhejiang NHU, NEPG, Anhui Tiger Biotech, Xinfa Pharma,
Kemin, Corbion, Jungbunzlauer, TotalEnergies Corbion, Novamont, Braskem,
Danimer/Teknor Apex, Amyris, POET, Green Plains, Raízen, Verbio, Quorn
Foods, Perfect Day, Solar Foods, and Calysta/Calysseo. Also includes
auth and admin panel improvements accumulated since last push.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NorthAmerica_biomanufacturing_database.xlsx
+++ b/data/NorthAmerica_biomanufacturing_database.xlsx
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U77"/>
+  <dimension ref="A1:U82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7005,6 +7005,331 @@
       <c r="T77" s="3" t="inlineStr"/>
       <c r="U77" s="3" t="inlineStr"/>
     </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>5013</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>dsm-firmenich Kingstree</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Captive</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Kingstree</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>DSM Nutritional Products site in Kingstree, South Carolina, producing carotenoids including canthaxanthin and beta-carotene through fermentation-derived and synthetic-route processes for the animal nutrition, aquaculture and food colouring markets. Canthaxanthin is used as a pigmenting agent in salmon, trout and poultry feed. Part of dsm-firmenich's Animal Nutrition &amp; Health division.</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>Microbial fermentation
+Fermentation (industrial)
+Downstream processing</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Carotenoid synthesis and fermentation-derived routes
+Canthaxanthin and beta-carotene production
+Encapsulation for feed applications
+Nutritional ingredient formulation</t>
+        </is>
+      </c>
+      <c r="M78" t="n">
+        <v>4</v>
+      </c>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>ISO 9001
+ISO 14001
+FAMI-QS</t>
+        </is>
+      </c>
+      <c r="Q78" t="inlineStr">
+        <is>
+          <t>Produces canthaxanthin for salmon/trout aquaculture pigmentation and poultry skin colour. Part of dsm-firmenich Animal Nutrition &amp; Health.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>5014</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>dsm-firmenich Newark</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Captive</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Newark</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>Flavour and fragrance manufacturing facility of dsm-firmenich (Firmenich heritage) at 150 Firmenich Way, Newark, New Jersey. Produces encapsulated flavours for food and beverage applications, fragrance ingredients for personal care, and taste molecules for consumer products. Serves as a key North American production hub for the Perfumery, Beauty &amp; Care and Taste, Texture &amp; Health divisions. ~100 employees on site.</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>Microbial fermentation
+Enzymatic catalysis
+Fermentation (industrial)</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Encapsulated flavour manufacturing
+Fermentation-derived taste molecules
+Fragrance ingredient production
+Spray-dried flavour encapsulation</t>
+        </is>
+      </c>
+      <c r="M79" t="n">
+        <v>4</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>ISO 9001
+ISO 22000
+FSSC 22000</t>
+        </is>
+      </c>
+      <c r="Q79" t="inlineStr">
+        <is>
+          <t>Firmenich heritage site at 150 Firmenich Way, Newark NJ. ~100 employees. North American production hub for dsm-firmenich flavour and fragrance divisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>5015</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>dsm-firmenich Plainsboro – Food &amp; Beverage Pilot</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Pilot facility</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Plainsboro</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Food &amp; Beverage co-creation and scale-up pilot facility opened March 2024 at the dsm-firmenich North America innovation campus in Plainsboro, New Jersey. Enables customers to develop and scale fermentation-derived flavours, functional food ingredients, texture systems and health ingredients in collaboration with dsm-firmenich application scientists. Houses pilot fermentation, formulation labs and sensory evaluation suites.</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Microbial fermentation
+Enzymatic catalysis
+Fermentation (industrial)</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Pilot fermentation for taste and flavour molecules
+Functional ingredient formulation and texturisation
+Sensory evaluation and application testing
+Scale-up from bench to pilot for food &amp; beverage customers</t>
+        </is>
+      </c>
+      <c r="M80" t="n">
+        <v>4</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>ISO 9001
+ISO 22000</t>
+        </is>
+      </c>
+      <c r="Q80" t="inlineStr">
+        <is>
+          <t>Opened March 2024. Co-creation model: customers develop and scale innovations with dsm-firmenich scientists on-site. Part of Plainsboro North America innovation campus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>5016</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>dsm-firmenich Schenectady</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Captive</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Schenectady</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>Nutritional premix and ingredient blending facility in Schenectady, New York, established 1995. Produces vitamin and mineral premixes, nutritional blends and customised ingredient solutions for food fortification, dietary supplements and animal nutrition customers. Underwent a $10 million production modernisation and audit-readiness upgrade completed in 2024–2025, adding automation and traceability systems.</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Fermentation (industrial)
+Downstream processing</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Vitamin and mineral premix blending
+Custom nutritional blend formulation
+Micronutrient encapsulation and coating
+Automated batch assembly and traceability</t>
+        </is>
+      </c>
+      <c r="M81" t="n">
+        <v>4</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>ISO 9001
+ISO 22000
+FSSC 22000
+NSF
+HACCP</t>
+        </is>
+      </c>
+      <c r="Q81" t="inlineStr">
+        <is>
+          <t>Established 1995. $10M modernisation upgrade 2024–2025. Nutritional premix hub for dsm-firmenich North America Health, Nutrition &amp; Care division.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>5017</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>dsm-firmenich Tonganoxie – NextGen Pet Nutrition</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Captive</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Tonganoxie</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>https://www.dsm-firmenich.com</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>Fully automated pet nutrition premix manufacturing facility ('NextGen Tonganoxie') opened October 2025 in Kansas. Dedicated exclusively to pet food nutrition, featuring 100% automated micro-ingredient addition systems, fully traceable batch assembly and advanced quality control. Produces highly customised vitamin, mineral and amino acid premixes for pet food manufacturers. Part of dsm-firmenich's Animal Nutrition &amp; Health pet segment.</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Fermentation (industrial)
+Downstream processing</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Automated micro-ingredient dosing and blending
+Fermentation-derived amino acid premix incorporation
+100% traceable batch assembly system
+Custom pet nutrition premix manufacturing</t>
+        </is>
+      </c>
+      <c r="M82" t="n">
+        <v>4</v>
+      </c>
+      <c r="N82" t="inlineStr">
+        <is>
+          <t>ISO 9001
+ISO 22000
+FSSC 22000
+FAMI-QS</t>
+        </is>
+      </c>
+      <c r="Q82" t="inlineStr">
+        <is>
+          <t>Opened October 2025. 100% automated micro-ingredient addition. Fully traceable. dsm-firmenich's dedicated NextGen pet nutrition manufacturing facility.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>